<commit_message>
Update case data, visualizations, and resources - 2025/12/01
</commit_message>
<xml_diff>
--- a/涉华投资仲裁案例统计总表（updated 251126）_KeerHuang.xlsx
+++ b/涉华投资仲裁案例统计总表（updated 251126）_KeerHuang.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0 科研材料\【工作】2024废物上工\Z中心和公众号事宜\【项目】涉华投资仲裁案例实时跟踪\涉华ISDS案件可视化 v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6269AEED-9D66-442E-B2AD-A1BB2971EC21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57B02560-0C79-44E4-B40D-4EBA09C16CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cases initiated by PRC investor" sheetId="1" r:id="rId1"/>
@@ -32923,7 +32923,7 @@
         <v>375</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>133</v>
+        <v>364</v>
       </c>
       <c r="S4" s="4"/>
       <c r="T4" s="6"/>

</xml_diff>